<commit_message>
Fix class-separated workbook structure
</commit_message>
<xml_diff>
--- a/Daftar_Siswa_Kelas_XI_2026_2027.xlsx
+++ b/Daftar_Siswa_Kelas_XI_2026_2027.xlsx
@@ -20,7 +20,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -42,7 +41,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="D9F1E1"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -70,7 +68,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="10"/>
@@ -1110,7 +1108,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="10"/>
@@ -2150,7 +2148,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="10"/>
@@ -3190,7 +3188,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="10"/>
@@ -4230,7 +4228,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="10"/>
@@ -5270,7 +5268,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="10"/>
@@ -6310,7 +6308,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="10"/>
@@ -7350,7 +7348,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="10"/>
@@ -8390,7 +8388,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="10"/>
@@ -9430,7 +9428,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="10"/>
@@ -10470,7 +10468,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="10"/>
@@ -11483,7 +11481,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="10"/>

</xml_diff>